<commit_message>
Auto update ETF comparison: Wed Jun 10 10:39:50 UTC 2026
</commit_message>
<xml_diff>
--- a/data/00403A/20260610.xlsx
+++ b/data/00403A/20260610.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="222">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="219">
   <si>
     <t xml:space="preserve">資料日期：115/06/10</t>
   </si>
@@ -71,9 +71,6 @@
     <t xml:space="preserve">NTD 6,404,084,696</t>
   </si>
   <si>
-    <t xml:space="preserve">3.71%</t>
-  </si>
-  <si>
     <t xml:space="preserve">期貨保證金</t>
   </si>
   <si>
@@ -83,16 +80,10 @@
     <t xml:space="preserve">NTD 15,074,362,032</t>
   </si>
   <si>
-    <t xml:space="preserve">8.73%</t>
-  </si>
-  <si>
     <t xml:space="preserve">應收付證券款</t>
   </si>
   <si>
     <t xml:space="preserve">NTD -2,240,533,576</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-1.30%</t>
   </si>
   <si>
     <t xml:space="preserve">股票代號</t>
@@ -1542,9 +1533,7 @@
       <c r="B12" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C12" s="2" t="s">
-        <v>10</v>
-      </c>
+      <c r="C12" s="2"/>
     </row>
     <row r="13">
       <c r="A13" s="19" t="s">
@@ -1553,42 +1542,34 @@
       <c r="B13" s="20" t="s">
         <v>18</v>
       </c>
-      <c r="C13" s="21" t="s">
-        <v>19</v>
-      </c>
+      <c r="C13" s="21"/>
     </row>
     <row r="14">
       <c r="A14" s="22" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B14" s="23" t="s">
         <v>12</v>
       </c>
-      <c r="C14" s="24" t="s">
-        <v>13</v>
-      </c>
+      <c r="C14" s="24"/>
     </row>
     <row r="15">
       <c r="A15" s="25" t="s">
+        <v>20</v>
+      </c>
+      <c r="B15" s="26" t="s">
         <v>21</v>
       </c>
-      <c r="B15" s="26" t="s">
-        <v>22</v>
-      </c>
-      <c r="C15" s="27" t="s">
-        <v>23</v>
-      </c>
+      <c r="C15" s="27"/>
     </row>
     <row r="16">
       <c r="A16" s="28" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B16" s="29" t="s">
-        <v>25</v>
-      </c>
-      <c r="C16" s="30" t="s">
-        <v>26</v>
-      </c>
+        <v>23</v>
+      </c>
+      <c r="C16" s="30"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="s">
@@ -1600,716 +1581,716 @@
     </row>
     <row r="20">
       <c r="A20" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D20" s="2" t="s">
         <v>27</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="B21" s="32" t="s">
+        <v>29</v>
+      </c>
+      <c r="C21" s="33" t="s">
+        <v>30</v>
+      </c>
+      <c r="D21" s="34" t="s">
         <v>31</v>
-      </c>
-      <c r="B21" s="32" t="s">
-        <v>32</v>
-      </c>
-      <c r="C21" s="33" t="s">
-        <v>33</v>
-      </c>
-      <c r="D21" s="34" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="35" t="s">
+        <v>32</v>
+      </c>
+      <c r="B22" s="36" t="s">
+        <v>33</v>
+      </c>
+      <c r="C22" s="37" t="s">
+        <v>34</v>
+      </c>
+      <c r="D22" s="38" t="s">
         <v>35</v>
-      </c>
-      <c r="B22" s="36" t="s">
-        <v>36</v>
-      </c>
-      <c r="C22" s="37" t="s">
-        <v>37</v>
-      </c>
-      <c r="D22" s="38" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="39" t="s">
+        <v>36</v>
+      </c>
+      <c r="B23" s="40" t="s">
+        <v>37</v>
+      </c>
+      <c r="C23" s="41" t="s">
+        <v>38</v>
+      </c>
+      <c r="D23" s="42" t="s">
         <v>39</v>
-      </c>
-      <c r="B23" s="40" t="s">
-        <v>40</v>
-      </c>
-      <c r="C23" s="41" t="s">
-        <v>41</v>
-      </c>
-      <c r="D23" s="42" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="43" t="s">
+        <v>40</v>
+      </c>
+      <c r="B24" s="44" t="s">
+        <v>41</v>
+      </c>
+      <c r="C24" s="45" t="s">
+        <v>42</v>
+      </c>
+      <c r="D24" s="46" t="s">
         <v>43</v>
-      </c>
-      <c r="B24" s="44" t="s">
-        <v>44</v>
-      </c>
-      <c r="C24" s="45" t="s">
-        <v>45</v>
-      </c>
-      <c r="D24" s="46" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="47" t="s">
+        <v>44</v>
+      </c>
+      <c r="B25" s="48" t="s">
+        <v>45</v>
+      </c>
+      <c r="C25" s="49" t="s">
+        <v>46</v>
+      </c>
+      <c r="D25" s="50" t="s">
         <v>47</v>
-      </c>
-      <c r="B25" s="48" t="s">
-        <v>48</v>
-      </c>
-      <c r="C25" s="49" t="s">
-        <v>49</v>
-      </c>
-      <c r="D25" s="50" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="51" t="s">
+        <v>48</v>
+      </c>
+      <c r="B26" s="52" t="s">
+        <v>49</v>
+      </c>
+      <c r="C26" s="53" t="s">
+        <v>50</v>
+      </c>
+      <c r="D26" s="54" t="s">
         <v>51</v>
-      </c>
-      <c r="B26" s="52" t="s">
-        <v>52</v>
-      </c>
-      <c r="C26" s="53" t="s">
-        <v>53</v>
-      </c>
-      <c r="D26" s="54" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="55" t="s">
+        <v>52</v>
+      </c>
+      <c r="B27" s="56" t="s">
+        <v>53</v>
+      </c>
+      <c r="C27" s="57" t="s">
+        <v>54</v>
+      </c>
+      <c r="D27" s="58" t="s">
         <v>55</v>
-      </c>
-      <c r="B27" s="56" t="s">
-        <v>56</v>
-      </c>
-      <c r="C27" s="57" t="s">
-        <v>57</v>
-      </c>
-      <c r="D27" s="58" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="59" t="s">
+        <v>56</v>
+      </c>
+      <c r="B28" s="60" t="s">
+        <v>57</v>
+      </c>
+      <c r="C28" s="61" t="s">
+        <v>58</v>
+      </c>
+      <c r="D28" s="62" t="s">
         <v>59</v>
-      </c>
-      <c r="B28" s="60" t="s">
-        <v>60</v>
-      </c>
-      <c r="C28" s="61" t="s">
-        <v>61</v>
-      </c>
-      <c r="D28" s="62" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="63" t="s">
+        <v>60</v>
+      </c>
+      <c r="B29" s="64" t="s">
+        <v>61</v>
+      </c>
+      <c r="C29" s="65" t="s">
+        <v>62</v>
+      </c>
+      <c r="D29" s="66" t="s">
         <v>63</v>
-      </c>
-      <c r="B29" s="64" t="s">
-        <v>64</v>
-      </c>
-      <c r="C29" s="65" t="s">
-        <v>65</v>
-      </c>
-      <c r="D29" s="66" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="67" t="s">
+        <v>64</v>
+      </c>
+      <c r="B30" s="68" t="s">
+        <v>65</v>
+      </c>
+      <c r="C30" s="69" t="s">
+        <v>66</v>
+      </c>
+      <c r="D30" s="70" t="s">
         <v>67</v>
-      </c>
-      <c r="B30" s="68" t="s">
-        <v>68</v>
-      </c>
-      <c r="C30" s="69" t="s">
-        <v>69</v>
-      </c>
-      <c r="D30" s="70" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="71" t="s">
+        <v>68</v>
+      </c>
+      <c r="B31" s="72" t="s">
+        <v>69</v>
+      </c>
+      <c r="C31" s="73" t="s">
+        <v>70</v>
+      </c>
+      <c r="D31" s="74" t="s">
         <v>71</v>
-      </c>
-      <c r="B31" s="72" t="s">
-        <v>72</v>
-      </c>
-      <c r="C31" s="73" t="s">
-        <v>73</v>
-      </c>
-      <c r="D31" s="74" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="75" t="s">
+        <v>72</v>
+      </c>
+      <c r="B32" s="76" t="s">
+        <v>73</v>
+      </c>
+      <c r="C32" s="77" t="s">
+        <v>74</v>
+      </c>
+      <c r="D32" s="78" t="s">
         <v>75</v>
-      </c>
-      <c r="B32" s="76" t="s">
-        <v>76</v>
-      </c>
-      <c r="C32" s="77" t="s">
-        <v>77</v>
-      </c>
-      <c r="D32" s="78" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="79" t="s">
+        <v>76</v>
+      </c>
+      <c r="B33" s="80" t="s">
+        <v>77</v>
+      </c>
+      <c r="C33" s="81" t="s">
+        <v>78</v>
+      </c>
+      <c r="D33" s="82" t="s">
         <v>79</v>
-      </c>
-      <c r="B33" s="80" t="s">
-        <v>80</v>
-      </c>
-      <c r="C33" s="81" t="s">
-        <v>81</v>
-      </c>
-      <c r="D33" s="82" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="83" t="s">
+        <v>80</v>
+      </c>
+      <c r="B34" s="84" t="s">
+        <v>81</v>
+      </c>
+      <c r="C34" s="85" t="s">
+        <v>82</v>
+      </c>
+      <c r="D34" s="86" t="s">
         <v>83</v>
-      </c>
-      <c r="B34" s="84" t="s">
-        <v>84</v>
-      </c>
-      <c r="C34" s="85" t="s">
-        <v>85</v>
-      </c>
-      <c r="D34" s="86" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="87" t="s">
+        <v>84</v>
+      </c>
+      <c r="B35" s="88" t="s">
+        <v>85</v>
+      </c>
+      <c r="C35" s="89" t="s">
+        <v>86</v>
+      </c>
+      <c r="D35" s="90" t="s">
         <v>87</v>
-      </c>
-      <c r="B35" s="88" t="s">
-        <v>88</v>
-      </c>
-      <c r="C35" s="89" t="s">
-        <v>89</v>
-      </c>
-      <c r="D35" s="90" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="91" t="s">
+        <v>88</v>
+      </c>
+      <c r="B36" s="92" t="s">
+        <v>89</v>
+      </c>
+      <c r="C36" s="93" t="s">
+        <v>90</v>
+      </c>
+      <c r="D36" s="94" t="s">
         <v>91</v>
-      </c>
-      <c r="B36" s="92" t="s">
-        <v>92</v>
-      </c>
-      <c r="C36" s="93" t="s">
-        <v>93</v>
-      </c>
-      <c r="D36" s="94" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="95" t="s">
+        <v>92</v>
+      </c>
+      <c r="B37" s="96" t="s">
+        <v>93</v>
+      </c>
+      <c r="C37" s="97" t="s">
+        <v>94</v>
+      </c>
+      <c r="D37" s="98" t="s">
         <v>95</v>
-      </c>
-      <c r="B37" s="96" t="s">
-        <v>96</v>
-      </c>
-      <c r="C37" s="97" t="s">
-        <v>97</v>
-      </c>
-      <c r="D37" s="98" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="99" t="s">
+        <v>96</v>
+      </c>
+      <c r="B38" s="100" t="s">
+        <v>97</v>
+      </c>
+      <c r="C38" s="101" t="s">
+        <v>98</v>
+      </c>
+      <c r="D38" s="102" t="s">
         <v>99</v>
-      </c>
-      <c r="B38" s="100" t="s">
-        <v>100</v>
-      </c>
-      <c r="C38" s="101" t="s">
-        <v>101</v>
-      </c>
-      <c r="D38" s="102" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="103" t="s">
+        <v>100</v>
+      </c>
+      <c r="B39" s="104" t="s">
+        <v>101</v>
+      </c>
+      <c r="C39" s="105" t="s">
+        <v>102</v>
+      </c>
+      <c r="D39" s="106" t="s">
         <v>103</v>
-      </c>
-      <c r="B39" s="104" t="s">
-        <v>104</v>
-      </c>
-      <c r="C39" s="105" t="s">
-        <v>105</v>
-      </c>
-      <c r="D39" s="106" t="s">
-        <v>106</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="107" t="s">
+        <v>104</v>
+      </c>
+      <c r="B40" s="108" t="s">
+        <v>105</v>
+      </c>
+      <c r="C40" s="109" t="s">
+        <v>106</v>
+      </c>
+      <c r="D40" s="110" t="s">
         <v>107</v>
-      </c>
-      <c r="B40" s="108" t="s">
-        <v>108</v>
-      </c>
-      <c r="C40" s="109" t="s">
-        <v>109</v>
-      </c>
-      <c r="D40" s="110" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="111" t="s">
+        <v>108</v>
+      </c>
+      <c r="B41" s="112" t="s">
+        <v>109</v>
+      </c>
+      <c r="C41" s="113" t="s">
+        <v>110</v>
+      </c>
+      <c r="D41" s="114" t="s">
         <v>111</v>
-      </c>
-      <c r="B41" s="112" t="s">
-        <v>112</v>
-      </c>
-      <c r="C41" s="113" t="s">
-        <v>113</v>
-      </c>
-      <c r="D41" s="114" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="115" t="s">
+        <v>112</v>
+      </c>
+      <c r="B42" s="116" t="s">
+        <v>113</v>
+      </c>
+      <c r="C42" s="117" t="s">
+        <v>114</v>
+      </c>
+      <c r="D42" s="118" t="s">
         <v>115</v>
-      </c>
-      <c r="B42" s="116" t="s">
-        <v>116</v>
-      </c>
-      <c r="C42" s="117" t="s">
-        <v>117</v>
-      </c>
-      <c r="D42" s="118" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="119" t="s">
+        <v>116</v>
+      </c>
+      <c r="B43" s="120" t="s">
+        <v>117</v>
+      </c>
+      <c r="C43" s="121" t="s">
+        <v>118</v>
+      </c>
+      <c r="D43" s="122" t="s">
         <v>119</v>
-      </c>
-      <c r="B43" s="120" t="s">
-        <v>120</v>
-      </c>
-      <c r="C43" s="121" t="s">
-        <v>121</v>
-      </c>
-      <c r="D43" s="122" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="123" t="s">
+        <v>120</v>
+      </c>
+      <c r="B44" s="124" t="s">
+        <v>121</v>
+      </c>
+      <c r="C44" s="125" t="s">
+        <v>122</v>
+      </c>
+      <c r="D44" s="126" t="s">
         <v>123</v>
-      </c>
-      <c r="B44" s="124" t="s">
-        <v>124</v>
-      </c>
-      <c r="C44" s="125" t="s">
-        <v>125</v>
-      </c>
-      <c r="D44" s="126" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="127" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="B45" s="128" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="C45" s="129" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="D45" s="130" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="131" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="B46" s="132" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="C46" s="133" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="D46" s="134" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="135" t="s">
+        <v>130</v>
+      </c>
+      <c r="B47" s="136" t="s">
+        <v>131</v>
+      </c>
+      <c r="C47" s="137" t="s">
+        <v>132</v>
+      </c>
+      <c r="D47" s="138" t="s">
         <v>133</v>
-      </c>
-      <c r="B47" s="136" t="s">
-        <v>134</v>
-      </c>
-      <c r="C47" s="137" t="s">
-        <v>135</v>
-      </c>
-      <c r="D47" s="138" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="139" t="s">
+        <v>134</v>
+      </c>
+      <c r="B48" s="140" t="s">
+        <v>135</v>
+      </c>
+      <c r="C48" s="141" t="s">
+        <v>136</v>
+      </c>
+      <c r="D48" s="142" t="s">
         <v>137</v>
-      </c>
-      <c r="B48" s="140" t="s">
-        <v>138</v>
-      </c>
-      <c r="C48" s="141" t="s">
-        <v>139</v>
-      </c>
-      <c r="D48" s="142" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="143" t="s">
+        <v>138</v>
+      </c>
+      <c r="B49" s="144" t="s">
+        <v>139</v>
+      </c>
+      <c r="C49" s="145" t="s">
+        <v>140</v>
+      </c>
+      <c r="D49" s="146" t="s">
         <v>141</v>
-      </c>
-      <c r="B49" s="144" t="s">
-        <v>142</v>
-      </c>
-      <c r="C49" s="145" t="s">
-        <v>143</v>
-      </c>
-      <c r="D49" s="146" t="s">
-        <v>144</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="147" t="s">
+        <v>142</v>
+      </c>
+      <c r="B50" s="148" t="s">
+        <v>143</v>
+      </c>
+      <c r="C50" s="149" t="s">
+        <v>144</v>
+      </c>
+      <c r="D50" s="150" t="s">
         <v>145</v>
-      </c>
-      <c r="B50" s="148" t="s">
-        <v>146</v>
-      </c>
-      <c r="C50" s="149" t="s">
-        <v>147</v>
-      </c>
-      <c r="D50" s="150" t="s">
-        <v>148</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="151" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="B51" s="152" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="C51" s="153" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="D51" s="154" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="155" t="s">
+        <v>149</v>
+      </c>
+      <c r="B52" s="156" t="s">
+        <v>150</v>
+      </c>
+      <c r="C52" s="157" t="s">
+        <v>151</v>
+      </c>
+      <c r="D52" s="158" t="s">
         <v>152</v>
-      </c>
-      <c r="B52" s="156" t="s">
-        <v>153</v>
-      </c>
-      <c r="C52" s="157" t="s">
-        <v>154</v>
-      </c>
-      <c r="D52" s="158" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="159" t="s">
+        <v>153</v>
+      </c>
+      <c r="B53" s="160" t="s">
+        <v>154</v>
+      </c>
+      <c r="C53" s="161" t="s">
+        <v>155</v>
+      </c>
+      <c r="D53" s="162" t="s">
         <v>156</v>
-      </c>
-      <c r="B53" s="160" t="s">
-        <v>157</v>
-      </c>
-      <c r="C53" s="161" t="s">
-        <v>158</v>
-      </c>
-      <c r="D53" s="162" t="s">
-        <v>159</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="163" t="s">
+        <v>157</v>
+      </c>
+      <c r="B54" s="164" t="s">
+        <v>158</v>
+      </c>
+      <c r="C54" s="165" t="s">
+        <v>159</v>
+      </c>
+      <c r="D54" s="166" t="s">
         <v>160</v>
-      </c>
-      <c r="B54" s="164" t="s">
-        <v>161</v>
-      </c>
-      <c r="C54" s="165" t="s">
-        <v>162</v>
-      </c>
-      <c r="D54" s="166" t="s">
-        <v>163</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="167" t="s">
+        <v>161</v>
+      </c>
+      <c r="B55" s="168" t="s">
+        <v>162</v>
+      </c>
+      <c r="C55" s="169" t="s">
+        <v>163</v>
+      </c>
+      <c r="D55" s="170" t="s">
         <v>164</v>
-      </c>
-      <c r="B55" s="168" t="s">
-        <v>165</v>
-      </c>
-      <c r="C55" s="169" t="s">
-        <v>166</v>
-      </c>
-      <c r="D55" s="170" t="s">
-        <v>167</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="171" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="B56" s="172" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="C56" s="173" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="D56" s="174" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="175" t="s">
+        <v>168</v>
+      </c>
+      <c r="B57" s="176" t="s">
+        <v>169</v>
+      </c>
+      <c r="C57" s="177" t="s">
+        <v>170</v>
+      </c>
+      <c r="D57" s="178" t="s">
         <v>171</v>
-      </c>
-      <c r="B57" s="176" t="s">
-        <v>172</v>
-      </c>
-      <c r="C57" s="177" t="s">
-        <v>173</v>
-      </c>
-      <c r="D57" s="178" t="s">
-        <v>174</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="179" t="s">
+        <v>172</v>
+      </c>
+      <c r="B58" s="180" t="s">
+        <v>173</v>
+      </c>
+      <c r="C58" s="181" t="s">
+        <v>174</v>
+      </c>
+      <c r="D58" s="182" t="s">
         <v>175</v>
-      </c>
-      <c r="B58" s="180" t="s">
-        <v>176</v>
-      </c>
-      <c r="C58" s="181" t="s">
-        <v>177</v>
-      </c>
-      <c r="D58" s="182" t="s">
-        <v>178</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="183" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="B59" s="184" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="C59" s="185" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="D59" s="186" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="187" t="s">
+        <v>179</v>
+      </c>
+      <c r="B60" s="188" t="s">
+        <v>180</v>
+      </c>
+      <c r="C60" s="189" t="s">
+        <v>181</v>
+      </c>
+      <c r="D60" s="190" t="s">
         <v>182</v>
-      </c>
-      <c r="B60" s="188" t="s">
-        <v>183</v>
-      </c>
-      <c r="C60" s="189" t="s">
-        <v>184</v>
-      </c>
-      <c r="D60" s="190" t="s">
-        <v>185</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="191" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="B61" s="192" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="C61" s="193" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="D61" s="194" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="195" t="s">
+        <v>186</v>
+      </c>
+      <c r="B62" s="196" t="s">
+        <v>187</v>
+      </c>
+      <c r="C62" s="197" t="s">
+        <v>188</v>
+      </c>
+      <c r="D62" s="198" t="s">
         <v>189</v>
-      </c>
-      <c r="B62" s="196" t="s">
-        <v>190</v>
-      </c>
-      <c r="C62" s="197" t="s">
-        <v>191</v>
-      </c>
-      <c r="D62" s="198" t="s">
-        <v>192</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="199" t="s">
+        <v>190</v>
+      </c>
+      <c r="B63" s="200" t="s">
+        <v>191</v>
+      </c>
+      <c r="C63" s="201" t="s">
+        <v>192</v>
+      </c>
+      <c r="D63" s="202" t="s">
         <v>193</v>
-      </c>
-      <c r="B63" s="200" t="s">
-        <v>194</v>
-      </c>
-      <c r="C63" s="201" t="s">
-        <v>195</v>
-      </c>
-      <c r="D63" s="202" t="s">
-        <v>196</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="203" t="s">
+        <v>194</v>
+      </c>
+      <c r="B64" s="204" t="s">
+        <v>195</v>
+      </c>
+      <c r="C64" s="205" t="s">
+        <v>196</v>
+      </c>
+      <c r="D64" s="206" t="s">
         <v>197</v>
-      </c>
-      <c r="B64" s="204" t="s">
-        <v>198</v>
-      </c>
-      <c r="C64" s="205" t="s">
-        <v>199</v>
-      </c>
-      <c r="D64" s="206" t="s">
-        <v>200</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="207" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="B65" s="208" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="C65" s="209" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="D65" s="210" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="211" t="s">
+        <v>201</v>
+      </c>
+      <c r="B66" s="212" t="s">
+        <v>202</v>
+      </c>
+      <c r="C66" s="213" t="s">
+        <v>203</v>
+      </c>
+      <c r="D66" s="214" t="s">
         <v>204</v>
-      </c>
-      <c r="B66" s="212" t="s">
-        <v>205</v>
-      </c>
-      <c r="C66" s="213" t="s">
-        <v>206</v>
-      </c>
-      <c r="D66" s="214" t="s">
-        <v>207</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="215" t="s">
+        <v>205</v>
+      </c>
+      <c r="B67" s="216" t="s">
+        <v>206</v>
+      </c>
+      <c r="C67" s="217" t="s">
+        <v>207</v>
+      </c>
+      <c r="D67" s="218" t="s">
         <v>208</v>
-      </c>
-      <c r="B67" s="216" t="s">
-        <v>209</v>
-      </c>
-      <c r="C67" s="217" t="s">
-        <v>210</v>
-      </c>
-      <c r="D67" s="218" t="s">
-        <v>211</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="219" t="s">
+        <v>209</v>
+      </c>
+      <c r="B68" s="220" t="s">
+        <v>210</v>
+      </c>
+      <c r="C68" s="221" t="s">
+        <v>211</v>
+      </c>
+      <c r="D68" s="222" t="s">
         <v>212</v>
-      </c>
-      <c r="B68" s="220" t="s">
-        <v>213</v>
-      </c>
-      <c r="C68" s="221" t="s">
-        <v>214</v>
-      </c>
-      <c r="D68" s="222" t="s">
-        <v>215</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="223" t="s">
+        <v>213</v>
+      </c>
+      <c r="B69" s="224" t="s">
+        <v>214</v>
+      </c>
+      <c r="C69" s="225" t="s">
+        <v>215</v>
+      </c>
+      <c r="D69" s="226" t="s">
         <v>216</v>
-      </c>
-      <c r="B69" s="224" t="s">
-        <v>217</v>
-      </c>
-      <c r="C69" s="225" t="s">
-        <v>218</v>
-      </c>
-      <c r="D69" s="226" t="s">
-        <v>219</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="227" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="B70" s="228" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="C70" s="229" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="D70" s="230" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
     </row>
   </sheetData>
@@ -2318,6 +2299,11 @@
     <mergeCell ref="B4:C4"/>
     <mergeCell ref="B5:C5"/>
     <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="B16:C16"/>
     <mergeCell ref="A19:D19"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>